<commit_message>
TWY E Rev P08: cable spec per fitting, and circuit-level testing
One 2-core 4 sq.mm secondary cable serves each fitting, SBC and TCC alike -
7 No. SBC and 12 No. TCC, 19 No. runs. Named in the scope sequence (Phase 3,
item 4), in the quantities column header and basis panel, and in the material
workbook.

Testing and commissioning is stated as a circuit-level activity covering the
affected fittings together with the fittings on the same circuits that fall
outside these works, since the series circuits are proved end to end before
handover. Recorded in the scope sequence (Phase 3, item 6), on the 5-day
schedule and in the quantities exclusions, which also notes that no material is
allowed for those unaffected fittings.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VJQm9FRnDf8JGAAWEgrXR2
</commit_message>
<xml_diff>
--- a/skills/zia-mta-basemap/examples/twy-e-asbuilt-ducts/material/Material Requirement - TWY E AGL Installation - Rev P08.xlsx
+++ b/skills/zia-mta-basemap/examples/twy-e-asbuilt-ducts/material/Material Requirement - TWY E AGL Installation - Rev P08.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="56">
   <si>
     <t xml:space="preserve">MATERIAL REQUIREMENT — AGL INSTALLATION</t>
   </si>
@@ -139,7 +139,7 @@
     <t xml:space="preserve">mtr</t>
   </si>
   <si>
-    <t xml:space="preserve">Saw cut route length is approx. 420 m over 19 No. runs. 1500 m covers the full manhole-to-light runs (no joints) plus terminations and tails — confirm against the run-by-run lengths now that 19 No. runs are in scope.</t>
+    <t xml:space="preserve">1 No. 2-core 4 sq.mm cable to each fitting, SBC and TCC alike — 7 No. SBC and 12 No. TCC = 19 No. runs. Saw cut route length is approx. 420 m; 1500 m covers the full manhole-to-light runs (no joints) plus terminations and tails — confirm against the run-by-run lengths.</t>
   </si>
   <si>
     <t xml:space="preserve">Masking tape</t>
@@ -181,13 +181,16 @@
     <t xml:space="preserve">3.  Sealant, mortar and backer rod quantities depend on the saw cut width and depth and on the core diameter. Both are set by the saw cut &amp; side-entry shallow base detail drawing, which had not been issued at Rev P08 (hold point H5). Re-check these three lines when it is issued.</t>
   </si>
   <si>
-    <t xml:space="preserve">4.  Secondary cable is ordered against the full manhole-to-light runs (19 No.), not the saw cut length — the cut measures approx. 420 m across the three locations (approx. 300 m LOC-01, 24 m LOC-02, 95 m LOC-03).</t>
+    <t xml:space="preserve">4.  One 2-core 4 sq.mm secondary cable serves each fitting, SBC and TCC alike — 7 No. SBC and 12 No. TCC. Cable is ordered against the full manhole-to-light runs (19 No.), not the saw cut length — the cut measures approx. 420 m across the three locations (approx. 300 m LOC-01, 24 m LOC-02, 95 m LOC-03).</t>
   </si>
   <si>
     <t xml:space="preserve">5.  Saw cut is an interim arrangement agreed between the AGL team, the civil team and ADA AGL. Permanent duct provision follows under the South Rehabilitation works, and is not covered by this requirement.</t>
   </si>
   <si>
-    <t xml:space="preserve">6.  Remaining Qty is a formula (Required − Available). Edit only the Required and Available columns.</t>
+    <t xml:space="preserve">6.  Testing and commissioning is carried out at circuit level and covers the affected fittings together with the fittings on the same circuits that fall outside these works — the series circuits are proved end to end before handover.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.  Remaining Qty is a formula (Required − Available). Edit only the Required and Available columns.</t>
   </si>
 </sst>
 </file>
@@ -730,7 +733,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -1138,14 +1141,26 @@
       <c r="F29" s="27"/>
       <c r="G29" s="27"/>
     </row>
+    <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A30:G30"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>